<commit_message>
Add Airbnb candidate from link intake
</commit_message>
<xml_diff>
--- a/exports/costa-blanca-matrix.xlsx
+++ b/exports/costa-blanca-matrix.xlsx
@@ -17,12 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Crawl Status" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kandidaten'!$A$1:$AW$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bewertungsmatrix'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kandidaten'!$A$1:$AW$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bewertungsmatrix'!$A$1:$K$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ausgeschlossen'!$A$1:$AW$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Flüge'!$A$1:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Link Intake'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Raw Crawl Status'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Link Intake'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Raw Crawl Status'!$A$1:$K$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -258,8 +258,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidatesTable" displayName="CandidatesTable" ref="A1:AW11" headerRowCount="1">
-  <autoFilter ref="A1:AW11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidatesTable" displayName="CandidatesTable" ref="A1:AW12" headerRowCount="1">
+  <autoFilter ref="A1:AW12"/>
   <tableColumns count="49">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="status"/>
@@ -316,8 +316,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ScoringMatrixTable" displayName="ScoringMatrixTable" ref="A1:K11" headerRowCount="1">
-  <autoFilter ref="A1:K11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ScoringMatrixTable" displayName="ScoringMatrixTable" ref="A1:K12" headerRowCount="1">
+  <autoFilter ref="A1:K12"/>
   <tableColumns count="11">
     <tableColumn id="1" name="name"/>
     <tableColumn id="2" name="location"/>
@@ -407,8 +407,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="LinkIntakeTable" displayName="LinkIntakeTable" ref="A1:L3" headerRowCount="1">
-  <autoFilter ref="A1:L3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="LinkIntakeTable" displayName="LinkIntakeTable" ref="A1:L4" headerRowCount="1">
+  <autoFilter ref="A1:L4"/>
   <tableColumns count="12">
     <tableColumn id="1" name="link_id"/>
     <tableColumn id="2" name="status"/>
@@ -428,8 +428,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RawCrawlStatusTable" displayName="RawCrawlStatusTable" ref="A1:K13" headerRowCount="1">
-  <autoFilter ref="A1:K13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RawCrawlStatusTable" displayName="RawCrawlStatusTable" ref="A1:K15" headerRowCount="1">
+  <autoFilter ref="A1:K15"/>
   <tableColumns count="11">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="name"/>
@@ -801,11 +801,11 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="4" t="n">
@@ -813,7 +813,7 @@
       </c>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="n"/>
     </row>
@@ -1444,29 +1444,29 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Apartamento Saul de Tarso</t>
+          <t>Apartment mit Blick auf das Mittelmeer</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Beniarbeig</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>279.81</v>
+        <v>500</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>6.15</v>
+        <v>5.5</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/es/apartamento-saul.html</t>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
         </is>
       </c>
       <c r="H33" s="2" t="n"/>
@@ -1504,29 +1504,29 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Margarida holiday bungalow</t>
+          <t>Apartamento Saul de Tarso</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Benitatxell Cumbre</t>
+          <t>Beniarbeig</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>454.19</v>
+        <v>279.81</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>7.22</v>
+        <v>6.15</v>
       </c>
       <c r="E35" s="8" t="n">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/es/margarida-holiday-bungalow-in-peaceful-surroundings-in-benitachell.html</t>
+          <t>https://www.booking.com/hotel/es/apartamento-saul.html</t>
         </is>
       </c>
       <c r="H35" s="2" t="n"/>
@@ -1534,29 +1534,29 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Apartamento Benitachell en Cumbres del Sol</t>
+          <t>Margarida holiday bungalow</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Cumbre del Sol</t>
+          <t>Benitatxell Cumbre</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>441</v>
+        <v>454.19</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>6.72</v>
+        <v>7.22</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/es/pueblo-de-la-paz-el-poble-nou-de-benitatxell-benitachell.html</t>
+          <t>https://www.booking.com/hotel/es/margarida-holiday-bungalow-in-peaceful-surroundings-in-benitachell.html</t>
         </is>
       </c>
       <c r="H36" s="2" t="n"/>
@@ -1828,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW11"/>
+  <dimension ref="A1:AW12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4091,9 +4091,220 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>cand_01b1a36aa388</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>airbnb</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>airbnb</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Apartment mit Blick auf das Mittelmeer</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>8 nights (user-provided)</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>apartment</t>
+        </is>
+      </c>
+      <c r="S12" s="12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="T12" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="U12" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="V12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y12" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z12" s="12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="AA12" s="12" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AC12" s="12" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AD12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AE12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AF12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AH12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AK12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AL12" s="13" t="inlineStr"/>
+      <c r="AM12" s="13" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN12" s="13" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AO12" s="8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AP12" s="8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AQ12" s="8" t="inlineStr">
+        <is>
+          <t>data/raw/link_01b1a36aa388.md</t>
+        </is>
+      </c>
+      <c r="AR12" s="8" t="inlineStr">
+        <is>
+          <t>data/raw/link_01b1a36aa388.json</t>
+        </is>
+      </c>
+      <c r="AS12" s="8" t="inlineStr"/>
+      <c r="AT12" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AU12" s="13" t="inlineStr"/>
+      <c r="AV12" s="13" t="inlineStr">
+        <is>
+          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
+        </is>
+      </c>
+      <c r="AW12" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AW11"/>
-  <conditionalFormatting sqref="Z2:Z11">
+  <autoFilter ref="A1:AW12"/>
+  <conditionalFormatting sqref="Z2:Z12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4105,7 +4316,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T11">
+  <conditionalFormatting sqref="T2:T12">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4117,7 +4328,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O11">
+  <conditionalFormatting sqref="O2:O12">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
       <formula>"true"</formula>
     </cfRule>
@@ -4125,7 +4336,7 @@
       <formula>"false"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT2:AT11">
+  <conditionalFormatting sqref="AT2:AT12">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
       <formula>"true"</formula>
     </cfRule>
@@ -4141,10 +4352,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4155,7 +4367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4638,9 +4850,50 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Apartment mit Blick auf das Mittelmeer</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
-  <conditionalFormatting sqref="J2:J11">
+  <autoFilter ref="A1:K12"/>
+  <conditionalFormatting sqref="J2:J12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4652,7 +4905,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D11">
+  <conditionalFormatting sqref="D2:D12">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5710,7 +5963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5857,8 +6110,70 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>link_01b1a36aa388</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Mati</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>airbnb</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>8 nights, user note: ca. 500 EUR pp</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights.</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6044,7 +6359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6488,17 +6803,41 @@
       <c r="K11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr"/>
-      <c r="B12" s="8" t="inlineStr"/>
-      <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>cand_01b1a36aa388</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Apartment mit Blick auf das Mittelmeer</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>data/raw/link_01b1a36aa388.md</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>data/raw/link_01b1a36aa388.json</t>
+        </is>
+      </c>
       <c r="H12" s="8" t="inlineStr"/>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -6506,11 +6845,7 @@
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr"/>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
+      <c r="K12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr"/>
@@ -6537,8 +6872,70 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr"/>
+      <c r="B14" s="8" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr"/>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>link_01b1a36aa388</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
+  <autoFilter ref="A1:K15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -6550,10 +6947,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add crawler handoff payloads for google sheet workflow
</commit_message>
<xml_diff>
--- a/exports/costa-blanca-matrix.xlsx
+++ b/exports/costa-blanca-matrix.xlsx
@@ -17,12 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Crawl Status" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kandidaten'!$A$1:$AW$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kandidaten'!$A$1:$AZ$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bewertungsmatrix'!$A$1:$K$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ausgeschlossen'!$A$1:$AW$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ausgeschlossen'!$A$1:$AZ$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Flüge'!$A$1:$D$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Link Intake'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Raw Crawl Status'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Raw Crawl Status'!$A$1:$N$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="€#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +68,23 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Aptos Display"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -96,8 +111,23 @@
         <fgColor rgb="002F6F73"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004D9078"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2B84B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D86F45"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -106,6 +136,20 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="00D7DEE2"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D7DEE2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D7DEE2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7DEE2"/>
+      </top>
       <bottom style="thin">
         <color rgb="00D7DEE2"/>
       </bottom>
@@ -120,7 +164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -149,7 +193,55 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,9 +350,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidatesTable" displayName="CandidatesTable" ref="A1:AW12" headerRowCount="1">
-  <autoFilter ref="A1:AW12"/>
-  <tableColumns count="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidatesTable" displayName="CandidatesTable" ref="A1:AZ12" headerRowCount="1">
+  <autoFilter ref="A1:AZ12"/>
+  <tableColumns count="52">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="status"/>
     <tableColumn id="3" name="source"/>
@@ -304,12 +396,15 @@
     <tableColumn id="41" name="crawl_status"/>
     <tableColumn id="42" name="needs_manual_input"/>
     <tableColumn id="43" name="raw_markdown_path"/>
-    <tableColumn id="44" name="raw_json_path"/>
-    <tableColumn id="45" name="screenshot_path"/>
-    <tableColumn id="46" name="excluded"/>
-    <tableColumn id="47" name="exclusion_reason"/>
-    <tableColumn id="48" name="notes"/>
-    <tableColumn id="49" name="last_updated"/>
+    <tableColumn id="44" name="raw_html_path"/>
+    <tableColumn id="45" name="raw_json_path"/>
+    <tableColumn id="46" name="extracted_json_path"/>
+    <tableColumn id="47" name="sheet_payload_path"/>
+    <tableColumn id="48" name="screenshot_path"/>
+    <tableColumn id="49" name="excluded"/>
+    <tableColumn id="50" name="exclusion_reason"/>
+    <tableColumn id="51" name="notes"/>
+    <tableColumn id="52" name="last_updated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -336,9 +431,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExcludedTable" displayName="ExcludedTable" ref="A1:AW4" headerRowCount="1">
-  <autoFilter ref="A1:AW4"/>
-  <tableColumns count="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExcludedTable" displayName="ExcludedTable" ref="A1:AZ4" headerRowCount="1">
+  <autoFilter ref="A1:AZ4"/>
+  <tableColumns count="52">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="status"/>
     <tableColumn id="3" name="source"/>
@@ -382,12 +477,15 @@
     <tableColumn id="41" name="crawl_status"/>
     <tableColumn id="42" name="needs_manual_input"/>
     <tableColumn id="43" name="raw_markdown_path"/>
-    <tableColumn id="44" name="raw_json_path"/>
-    <tableColumn id="45" name="screenshot_path"/>
-    <tableColumn id="46" name="excluded"/>
-    <tableColumn id="47" name="exclusion_reason"/>
-    <tableColumn id="48" name="notes"/>
-    <tableColumn id="49" name="last_updated"/>
+    <tableColumn id="44" name="raw_html_path"/>
+    <tableColumn id="45" name="raw_json_path"/>
+    <tableColumn id="46" name="extracted_json_path"/>
+    <tableColumn id="47" name="sheet_payload_path"/>
+    <tableColumn id="48" name="screenshot_path"/>
+    <tableColumn id="49" name="excluded"/>
+    <tableColumn id="50" name="exclusion_reason"/>
+    <tableColumn id="51" name="notes"/>
+    <tableColumn id="52" name="last_updated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -428,20 +526,23 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RawCrawlStatusTable" displayName="RawCrawlStatusTable" ref="A1:K15" headerRowCount="1">
-  <autoFilter ref="A1:K15"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RawCrawlStatusTable" displayName="RawCrawlStatusTable" ref="A1:N15" headerRowCount="1">
+  <autoFilter ref="A1:N15"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="name"/>
     <tableColumn id="3" name="url"/>
     <tableColumn id="4" name="crawl_status"/>
     <tableColumn id="5" name="needs_manual_input"/>
     <tableColumn id="6" name="raw_markdown_path"/>
-    <tableColumn id="7" name="raw_json_path"/>
-    <tableColumn id="8" name="screenshot_path"/>
-    <tableColumn id="9" name="last_updated"/>
-    <tableColumn id="10" name="link_id"/>
-    <tableColumn id="11" name="status"/>
+    <tableColumn id="7" name="raw_html_path"/>
+    <tableColumn id="8" name="raw_json_path"/>
+    <tableColumn id="9" name="extracted_json_path"/>
+    <tableColumn id="10" name="sheet_payload_path"/>
+    <tableColumn id="11" name="screenshot_path"/>
+    <tableColumn id="12" name="last_updated"/>
+    <tableColumn id="13" name="link_id"/>
+    <tableColumn id="14" name="status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -736,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -813,7 +914,7 @@
       </c>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="n"/>
     </row>
@@ -1783,13 +1884,212 @@
       </c>
       <c r="H45" s="2" t="n"/>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Crawler handoff</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Link intake &gt; Crawl &gt; Score &gt; Google Sheet payload</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>LINK</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>CRAWL</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>SCORE</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>SHEET</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="n"/>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>Intake</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>Raw HTML/MD</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Matrix</t>
+        </is>
+      </c>
+      <c r="D53" s="23" t="inlineStr">
+        <is>
+          <t>Payload JSON</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="inlineStr">
+        <is>
+          <t>Success crawls</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="24" t="inlineStr">
+        <is>
+          <t>Payloads ready</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
+          <t>Manual input</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="15">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="E7:H9"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A56:C56"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A55:C55"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="G3:H3"/>
@@ -1828,7 +2128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW12"/>
+  <dimension ref="A1:AZ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1874,256 +2174,274 @@
     <col width="15" customWidth="1" min="41" max="41"/>
     <col width="21" customWidth="1" min="42" max="42"/>
     <col width="34" customWidth="1" min="43" max="43"/>
-    <col width="34" customWidth="1" min="44" max="44"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
     <col width="34" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
-    <col width="42" customWidth="1" min="48" max="48"/>
-    <col width="15" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="46" max="46"/>
+    <col width="21" customWidth="1" min="47" max="47"/>
+    <col width="34" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="19" customWidth="1" min="50" max="50"/>
+    <col width="42" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>date_range</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>nights</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>lng</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="26" t="inlineStr">
         <is>
           <t>price_total</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="26" t="inlineStr">
         <is>
           <t>price_per_person</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="26" t="inlineStr">
         <is>
           <t>price_per_person_per_night</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="26" t="inlineStr">
         <is>
           <t>budget_under_500pp</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="P1" s="26" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="Q1" s="26" t="inlineStr">
         <is>
           <t>review_count</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="R1" s="26" t="inlineStr">
         <is>
           <t>property_type</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="S1" s="26" t="inlineStr">
         <is>
           <t>private_level</t>
         </is>
       </c>
-      <c r="T1" s="10" t="inlineStr">
+      <c r="T1" s="26" t="inlineStr">
         <is>
           <t>child_potential_0_10</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="U1" s="26" t="inlineStr">
         <is>
           <t>quiet_score_0_10</t>
         </is>
       </c>
-      <c r="V1" s="10" t="inlineStr">
+      <c r="V1" s="26" t="inlineStr">
         <is>
           <t>review_evidence_0_10</t>
         </is>
       </c>
-      <c r="W1" s="10" t="inlineStr">
+      <c r="W1" s="26" t="inlineStr">
         <is>
           <t>beach_fit_0_10</t>
         </is>
       </c>
-      <c r="X1" s="10" t="inlineStr">
+      <c r="X1" s="26" t="inlineStr">
         <is>
           <t>transfer_score_0_10</t>
         </is>
       </c>
-      <c r="Y1" s="10" t="inlineStr">
+      <c r="Y1" s="26" t="inlineStr">
         <is>
           <t>budget_score_0_10</t>
         </is>
       </c>
-      <c r="Z1" s="10" t="inlineStr">
+      <c r="Z1" s="26" t="inlineStr">
         <is>
           <t>overall_score_0_10</t>
         </is>
       </c>
-      <c r="AA1" s="10" t="inlineStr">
+      <c r="AA1" s="26" t="inlineStr">
         <is>
           <t>alc_km_est</t>
         </is>
       </c>
-      <c r="AB1" s="10" t="inlineStr">
+      <c r="AB1" s="26" t="inlineStr">
         <is>
           <t>alc_drive_min_est</t>
         </is>
       </c>
-      <c r="AC1" s="10" t="inlineStr">
+      <c r="AC1" s="26" t="inlineStr">
         <is>
           <t>vlc_km_est</t>
         </is>
       </c>
-      <c r="AD1" s="10" t="inlineStr">
+      <c r="AD1" s="26" t="inlineStr">
         <is>
           <t>vlc_drive_min_est</t>
         </is>
       </c>
-      <c r="AE1" s="10" t="inlineStr">
+      <c r="AE1" s="26" t="inlineStr">
         <is>
           <t>airport_distance_method</t>
         </is>
       </c>
-      <c r="AF1" s="10" t="inlineStr">
+      <c r="AF1" s="26" t="inlineStr">
         <is>
           <t>pool_type</t>
         </is>
       </c>
-      <c r="AG1" s="10" t="inlineStr">
+      <c r="AG1" s="26" t="inlineStr">
         <is>
           <t>whole_place_evidence</t>
         </is>
       </c>
-      <c r="AH1" s="10" t="inlineStr">
+      <c r="AH1" s="26" t="inlineStr">
         <is>
           <t>kitchen</t>
         </is>
       </c>
-      <c r="AI1" s="10" t="inlineStr">
+      <c r="AI1" s="26" t="inlineStr">
         <is>
           <t>air_conditioning</t>
         </is>
       </c>
-      <c r="AJ1" s="10" t="inlineStr">
+      <c r="AJ1" s="26" t="inlineStr">
         <is>
           <t>parking</t>
         </is>
       </c>
-      <c r="AK1" s="10" t="inlineStr">
+      <c r="AK1" s="26" t="inlineStr">
         <is>
           <t>terrace_or_balcony</t>
         </is>
       </c>
-      <c r="AL1" s="10" t="inlineStr">
+      <c r="AL1" s="26" t="inlineStr">
         <is>
           <t>family_red_flags</t>
         </is>
       </c>
-      <c r="AM1" s="10" t="inlineStr">
+      <c r="AM1" s="26" t="inlineStr">
         <is>
           <t>quiet_evidence</t>
         </is>
       </c>
-      <c r="AN1" s="10" t="inlineStr">
+      <c r="AN1" s="26" t="inlineStr">
         <is>
           <t>review_evidence</t>
         </is>
       </c>
-      <c r="AO1" s="10" t="inlineStr">
+      <c r="AO1" s="26" t="inlineStr">
         <is>
           <t>crawl_status</t>
         </is>
       </c>
-      <c r="AP1" s="10" t="inlineStr">
+      <c r="AP1" s="26" t="inlineStr">
         <is>
           <t>needs_manual_input</t>
         </is>
       </c>
-      <c r="AQ1" s="10" t="inlineStr">
+      <c r="AQ1" s="26" t="inlineStr">
         <is>
           <t>raw_markdown_path</t>
         </is>
       </c>
-      <c r="AR1" s="10" t="inlineStr">
+      <c r="AR1" s="26" t="inlineStr">
+        <is>
+          <t>raw_html_path</t>
+        </is>
+      </c>
+      <c r="AS1" s="26" t="inlineStr">
         <is>
           <t>raw_json_path</t>
         </is>
       </c>
-      <c r="AS1" s="10" t="inlineStr">
+      <c r="AT1" s="26" t="inlineStr">
+        <is>
+          <t>extracted_json_path</t>
+        </is>
+      </c>
+      <c r="AU1" s="26" t="inlineStr">
+        <is>
+          <t>sheet_payload_path</t>
+        </is>
+      </c>
+      <c r="AV1" s="26" t="inlineStr">
         <is>
           <t>screenshot_path</t>
         </is>
       </c>
-      <c r="AT1" s="10" t="inlineStr">
+      <c r="AW1" s="26" t="inlineStr">
         <is>
           <t>excluded</t>
         </is>
       </c>
-      <c r="AU1" s="10" t="inlineStr">
+      <c r="AX1" s="26" t="inlineStr">
         <is>
           <t>exclusion_reason</t>
         </is>
       </c>
-      <c r="AV1" s="10" t="inlineStr">
+      <c r="AY1" s="26" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="AW1" s="10" t="inlineStr">
+      <c r="AZ1" s="26" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -2183,13 +2501,13 @@
           <t>-0.005844</t>
         </is>
       </c>
-      <c r="L2" s="11" t="n">
+      <c r="L2" s="27" t="n">
         <v>559.62</v>
       </c>
-      <c r="M2" s="11" t="n">
+      <c r="M2" s="27" t="n">
         <v>279.81</v>
       </c>
-      <c r="N2" s="11" t="n">
+      <c r="N2" s="27" t="n">
         <v>31.09</v>
       </c>
       <c r="O2" s="8" t="inlineStr">
@@ -2212,37 +2530,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S2" s="12" t="n">
+      <c r="S2" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="T2" s="12" t="n">
+      <c r="T2" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="U2" s="12" t="n">
+      <c r="U2" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="V2" s="12" t="n">
+      <c r="V2" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="W2" s="12" t="n">
+      <c r="W2" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="X2" s="12" t="n">
+      <c r="X2" s="28" t="n">
         <v>6.5</v>
       </c>
-      <c r="Y2" s="12" t="n">
+      <c r="Y2" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="Z2" s="12" t="n">
+      <c r="Z2" s="28" t="n">
         <v>6.15</v>
       </c>
-      <c r="AA2" s="12" t="n">
+      <c r="AA2" s="28" t="n">
         <v>94.59999999999999</v>
       </c>
       <c r="AB2" s="8" t="n">
         <v>76</v>
       </c>
-      <c r="AC2" s="12" t="n">
+      <c r="AC2" s="28" t="n">
         <v>104.2</v>
       </c>
       <c r="AD2" s="8" t="n">
@@ -2283,13 +2601,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL2" s="13" t="inlineStr"/>
-      <c r="AM2" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN2" s="13" t="inlineStr">
+      <c r="AL2" s="29" t="inlineStr"/>
+      <c r="AM2" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN2" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -2307,22 +2625,25 @@
       <c r="AQ2" s="8" t="inlineStr"/>
       <c r="AR2" s="8" t="inlineStr"/>
       <c r="AS2" s="8" t="inlineStr"/>
-      <c r="AT2" s="8" t="inlineStr">
+      <c r="AT2" s="8" t="inlineStr"/>
+      <c r="AU2" s="8" t="inlineStr"/>
+      <c r="AV2" s="8" t="inlineStr"/>
+      <c r="AW2" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU2" s="13" t="inlineStr">
+      <c r="AX2" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV2" s="13" t="inlineStr">
+      <c r="AY2" s="29" t="inlineStr">
         <is>
           <t>Budget fit but inland and weak beach profile</t>
         </is>
       </c>
-      <c r="AW2" s="8" t="inlineStr">
+      <c r="AZ2" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -2382,13 +2703,13 @@
           <t>-0.023002</t>
         </is>
       </c>
-      <c r="L3" s="11" t="n">
+      <c r="L3" s="27" t="n">
         <v>827.45</v>
       </c>
-      <c r="M3" s="11" t="n">
+      <c r="M3" s="27" t="n">
         <v>413.73</v>
       </c>
-      <c r="N3" s="11" t="n">
+      <c r="N3" s="27" t="n">
         <v>45.97</v>
       </c>
       <c r="O3" s="8" t="inlineStr">
@@ -2407,37 +2728,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S3" s="12" t="n">
+      <c r="S3" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="T3" s="12" t="n">
+      <c r="T3" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="U3" s="12" t="n">
+      <c r="U3" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="V3" s="12" t="n">
+      <c r="V3" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="W3" s="12" t="n">
+      <c r="W3" s="28" t="n">
         <v>7.4</v>
       </c>
-      <c r="X3" s="12" t="n">
+      <c r="X3" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="12" t="n">
+      <c r="Y3" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="Z3" s="12" t="n">
+      <c r="Z3" s="28" t="n">
         <v>6.83</v>
       </c>
-      <c r="AA3" s="12" t="n">
+      <c r="AA3" s="28" t="n">
         <v>75</v>
       </c>
       <c r="AB3" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="AC3" s="12" t="n">
+      <c r="AC3" s="28" t="n">
         <v>126.4</v>
       </c>
       <c r="AD3" s="8" t="n">
@@ -2478,13 +2799,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL3" s="13" t="inlineStr"/>
-      <c r="AM3" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN3" s="13" t="inlineStr">
+      <c r="AL3" s="29" t="inlineStr"/>
+      <c r="AM3" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN3" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -2502,22 +2823,25 @@
       <c r="AQ3" s="8" t="inlineStr"/>
       <c r="AR3" s="8" t="inlineStr"/>
       <c r="AS3" s="8" t="inlineStr"/>
-      <c r="AT3" s="8" t="inlineStr">
+      <c r="AT3" s="8" t="inlineStr"/>
+      <c r="AU3" s="8" t="inlineStr"/>
+      <c r="AV3" s="8" t="inlineStr"/>
+      <c r="AW3" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU3" s="13" t="inlineStr">
+      <c r="AX3" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV3" s="13" t="inlineStr">
+      <c r="AY3" s="29" t="inlineStr">
         <is>
           <t>Good Altea compromise but shared complex risk</t>
         </is>
       </c>
-      <c r="AW3" s="8" t="inlineStr">
+      <c r="AZ3" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -2577,13 +2901,13 @@
           <t>0.173084</t>
         </is>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="L4" s="27" t="n">
         <v>908.38</v>
       </c>
-      <c r="M4" s="11" t="n">
+      <c r="M4" s="27" t="n">
         <v>454.19</v>
       </c>
-      <c r="N4" s="11" t="n">
+      <c r="N4" s="27" t="n">
         <v>64.88</v>
       </c>
       <c r="O4" s="8" t="inlineStr">
@@ -2602,37 +2926,37 @@
           <t>holiday bungalow</t>
         </is>
       </c>
-      <c r="S4" s="12" t="n">
+      <c r="S4" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="T4" s="12" t="n">
+      <c r="T4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="U4" s="12" t="n">
+      <c r="U4" s="28" t="n">
         <v>8.5</v>
       </c>
-      <c r="V4" s="12" t="n">
+      <c r="V4" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="W4" s="12" t="n">
+      <c r="W4" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="X4" s="12" t="n">
+      <c r="X4" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="Y4" s="12" t="n">
+      <c r="Y4" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z4" s="12" t="n">
+      <c r="Z4" s="28" t="n">
         <v>7.22</v>
       </c>
-      <c r="AA4" s="12" t="n">
+      <c r="AA4" s="28" t="n">
         <v>98.40000000000001</v>
       </c>
       <c r="AB4" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="AC4" s="12" t="n">
+      <c r="AC4" s="28" t="n">
         <v>126.3</v>
       </c>
       <c r="AD4" s="8" t="n">
@@ -2673,13 +2997,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL4" s="13" t="inlineStr"/>
-      <c r="AM4" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN4" s="13" t="inlineStr">
+      <c r="AL4" s="29" t="inlineStr"/>
+      <c r="AM4" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN4" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -2697,22 +3021,25 @@
       <c r="AQ4" s="8" t="inlineStr"/>
       <c r="AR4" s="8" t="inlineStr"/>
       <c r="AS4" s="8" t="inlineStr"/>
-      <c r="AT4" s="8" t="inlineStr">
+      <c r="AT4" s="8" t="inlineStr"/>
+      <c r="AU4" s="8" t="inlineStr"/>
+      <c r="AV4" s="8" t="inlineStr"/>
+      <c r="AW4" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU4" s="13" t="inlineStr">
+      <c r="AX4" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV4" s="13" t="inlineStr">
+      <c r="AY4" s="29" t="inlineStr">
         <is>
           <t>Best cove profile under 1000 EUR if 7 nights okay</t>
         </is>
       </c>
-      <c r="AW4" s="8" t="inlineStr">
+      <c r="AZ4" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -2772,13 +3099,13 @@
           <t>0.172926</t>
         </is>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="27" t="n">
         <v>882</v>
       </c>
-      <c r="M5" s="11" t="n">
+      <c r="M5" s="27" t="n">
         <v>441</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="N5" s="27" t="n">
         <v>63</v>
       </c>
       <c r="O5" s="8" t="inlineStr">
@@ -2801,37 +3128,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S5" s="12" t="n">
+      <c r="S5" s="28" t="n">
         <v>5.8</v>
       </c>
-      <c r="T5" s="12" t="n">
+      <c r="T5" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="U5" s="12" t="n">
+      <c r="U5" s="28" t="n">
         <v>7.8</v>
       </c>
-      <c r="V5" s="12" t="n">
+      <c r="V5" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="W5" s="12" t="n">
+      <c r="W5" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="X5" s="12" t="n">
+      <c r="X5" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="Y5" s="12" t="n">
+      <c r="Y5" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="Z5" s="12" t="n">
+      <c r="Z5" s="28" t="n">
         <v>6.72</v>
       </c>
-      <c r="AA5" s="12" t="n">
+      <c r="AA5" s="28" t="n">
         <v>98.3</v>
       </c>
       <c r="AB5" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="AC5" s="12" t="n">
+      <c r="AC5" s="28" t="n">
         <v>126.4</v>
       </c>
       <c r="AD5" s="8" t="n">
@@ -2872,13 +3199,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL5" s="13" t="inlineStr"/>
-      <c r="AM5" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN5" s="13" t="inlineStr">
+      <c r="AL5" s="29" t="inlineStr"/>
+      <c r="AM5" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN5" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -2896,22 +3223,25 @@
       <c r="AQ5" s="8" t="inlineStr"/>
       <c r="AR5" s="8" t="inlineStr"/>
       <c r="AS5" s="8" t="inlineStr"/>
-      <c r="AT5" s="8" t="inlineStr">
+      <c r="AT5" s="8" t="inlineStr"/>
+      <c r="AU5" s="8" t="inlineStr"/>
+      <c r="AV5" s="8" t="inlineStr"/>
+      <c r="AW5" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU5" s="13" t="inlineStr">
+      <c r="AX5" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV5" s="13" t="inlineStr">
+      <c r="AY5" s="29" t="inlineStr">
         <is>
           <t>Strong Cumbre value but weak review evidence</t>
         </is>
       </c>
-      <c r="AW5" s="8" t="inlineStr">
+      <c r="AZ5" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -2971,13 +3301,13 @@
           <t>0.062501</t>
         </is>
       </c>
-      <c r="L6" s="11" t="n">
+      <c r="L6" s="27" t="n">
         <v>839.8</v>
       </c>
-      <c r="M6" s="11" t="n">
+      <c r="M6" s="27" t="n">
         <v>419.9</v>
       </c>
-      <c r="N6" s="11" t="n">
+      <c r="N6" s="27" t="n">
         <v>59.99</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
@@ -2996,37 +3326,37 @@
           <t>holiday home</t>
         </is>
       </c>
-      <c r="S6" s="12" t="n">
+      <c r="S6" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="T6" s="12" t="n">
+      <c r="T6" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="U6" s="12" t="n">
+      <c r="U6" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="V6" s="12" t="n">
+      <c r="V6" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="W6" s="12" t="n">
+      <c r="W6" s="28" t="n">
         <v>6.6</v>
       </c>
-      <c r="X6" s="12" t="n">
+      <c r="X6" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="Y6" s="12" t="n">
+      <c r="Y6" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="Z6" s="12" t="n">
+      <c r="Z6" s="28" t="n">
         <v>6.66</v>
       </c>
-      <c r="AA6" s="12" t="n">
+      <c r="AA6" s="28" t="n">
         <v>84.2</v>
       </c>
       <c r="AB6" s="8" t="n">
         <v>67</v>
       </c>
-      <c r="AC6" s="12" t="n">
+      <c r="AC6" s="28" t="n">
         <v>127.3</v>
       </c>
       <c r="AD6" s="8" t="n">
@@ -3067,13 +3397,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL6" s="13" t="inlineStr"/>
-      <c r="AM6" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN6" s="13" t="inlineStr">
+      <c r="AL6" s="29" t="inlineStr"/>
+      <c r="AM6" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN6" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -3091,22 +3421,25 @@
       <c r="AQ6" s="8" t="inlineStr"/>
       <c r="AR6" s="8" t="inlineStr"/>
       <c r="AS6" s="8" t="inlineStr"/>
-      <c r="AT6" s="8" t="inlineStr">
+      <c r="AT6" s="8" t="inlineStr"/>
+      <c r="AU6" s="8" t="inlineStr"/>
+      <c r="AV6" s="8" t="inlineStr"/>
+      <c r="AW6" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU6" s="13" t="inlineStr">
+      <c r="AX6" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV6" s="13" t="inlineStr">
+      <c r="AY6" s="29" t="inlineStr">
         <is>
           <t>Good price holiday home but only one review</t>
         </is>
       </c>
-      <c r="AW6" s="8" t="inlineStr">
+      <c r="AZ6" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -3166,13 +3499,13 @@
           <t>-0.103157</t>
         </is>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="27" t="n">
         <v>932.77</v>
       </c>
-      <c r="M7" s="11" t="n">
+      <c r="M7" s="27" t="n">
         <v>466.38</v>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="N7" s="27" t="n">
         <v>51.82</v>
       </c>
       <c r="O7" s="8" t="inlineStr">
@@ -3191,37 +3524,37 @@
           <t>holiday home</t>
         </is>
       </c>
-      <c r="S7" s="12" t="n">
+      <c r="S7" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="T7" s="12" t="n">
+      <c r="T7" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="U7" s="12" t="n">
+      <c r="U7" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="V7" s="12" t="n">
+      <c r="V7" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="W7" s="12" t="n">
+      <c r="W7" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="X7" s="12" t="n">
+      <c r="X7" s="28" t="n">
         <v>7.5</v>
       </c>
-      <c r="Y7" s="12" t="n">
+      <c r="Y7" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z7" s="12" t="n">
+      <c r="Z7" s="28" t="n">
         <v>6.96</v>
       </c>
-      <c r="AA7" s="12" t="n">
+      <c r="AA7" s="28" t="n">
         <v>74.5</v>
       </c>
       <c r="AB7" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="AC7" s="12" t="n">
+      <c r="AC7" s="28" t="n">
         <v>116</v>
       </c>
       <c r="AD7" s="8" t="n">
@@ -3262,13 +3595,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL7" s="13" t="inlineStr"/>
-      <c r="AM7" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN7" s="13" t="inlineStr">
+      <c r="AL7" s="29" t="inlineStr"/>
+      <c r="AM7" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN7" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -3286,22 +3619,25 @@
       <c r="AQ7" s="8" t="inlineStr"/>
       <c r="AR7" s="8" t="inlineStr"/>
       <c r="AS7" s="8" t="inlineStr"/>
-      <c r="AT7" s="8" t="inlineStr">
+      <c r="AT7" s="8" t="inlineStr"/>
+      <c r="AU7" s="8" t="inlineStr"/>
+      <c r="AV7" s="8" t="inlineStr"/>
+      <c r="AW7" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU7" s="13" t="inlineStr">
+      <c r="AX7" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV7" s="13" t="inlineStr">
+      <c r="AY7" s="29" t="inlineStr">
         <is>
           <t>Quiet and under budget but inland not beach fit</t>
         </is>
       </c>
-      <c r="AW7" s="8" t="inlineStr">
+      <c r="AZ7" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -3361,13 +3697,13 @@
           <t>0.172693</t>
         </is>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="27" t="n">
         <v>972</v>
       </c>
-      <c r="M8" s="11" t="n">
+      <c r="M8" s="27" t="n">
         <v>486</v>
       </c>
-      <c r="N8" s="11" t="n">
+      <c r="N8" s="27" t="n">
         <v>54</v>
       </c>
       <c r="O8" s="8" t="inlineStr">
@@ -3386,37 +3722,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S8" s="12" t="n">
+      <c r="S8" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="T8" s="12" t="n">
+      <c r="T8" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="U8" s="12" t="n">
+      <c r="U8" s="28" t="n">
         <v>7.8</v>
       </c>
-      <c r="V8" s="12" t="n">
+      <c r="V8" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="W8" s="12" t="n">
+      <c r="W8" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="X8" s="12" t="n">
+      <c r="X8" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="Y8" s="12" t="n">
+      <c r="Y8" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z8" s="12" t="n">
+      <c r="Z8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="AA8" s="12" t="n">
+      <c r="AA8" s="28" t="n">
         <v>98.40000000000001</v>
       </c>
       <c r="AB8" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="AC8" s="12" t="n">
+      <c r="AC8" s="28" t="n">
         <v>126.3</v>
       </c>
       <c r="AD8" s="8" t="n">
@@ -3457,13 +3793,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL8" s="13" t="inlineStr"/>
-      <c r="AM8" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN8" s="13" t="inlineStr">
+      <c r="AL8" s="29" t="inlineStr"/>
+      <c r="AM8" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN8" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -3481,22 +3817,25 @@
       <c r="AQ8" s="8" t="inlineStr"/>
       <c r="AR8" s="8" t="inlineStr"/>
       <c r="AS8" s="8" t="inlineStr"/>
-      <c r="AT8" s="8" t="inlineStr">
+      <c r="AT8" s="8" t="inlineStr"/>
+      <c r="AU8" s="8" t="inlineStr"/>
+      <c r="AV8" s="8" t="inlineStr"/>
+      <c r="AW8" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU8" s="13" t="inlineStr">
+      <c r="AX8" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV8" s="13" t="inlineStr">
+      <c r="AY8" s="29" t="inlineStr">
         <is>
           <t>Good location but excluded by prior detail-risk evidence</t>
         </is>
       </c>
-      <c r="AW8" s="8" t="inlineStr">
+      <c r="AZ8" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -3556,13 +3895,13 @@
           <t>0.075664</t>
         </is>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="27" t="n">
         <v>997</v>
       </c>
-      <c r="M9" s="11" t="n">
+      <c r="M9" s="27" t="n">
         <v>498.5</v>
       </c>
-      <c r="N9" s="11" t="n">
+      <c r="N9" s="27" t="n">
         <v>55.39</v>
       </c>
       <c r="O9" s="8" t="inlineStr">
@@ -3585,37 +3924,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S9" s="12" t="n">
+      <c r="S9" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="T9" s="12" t="n">
+      <c r="T9" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="U9" s="12" t="n">
+      <c r="U9" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="V9" s="12" t="n">
+      <c r="V9" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="W9" s="12" t="n">
+      <c r="W9" s="28" t="n">
         <v>3.5</v>
       </c>
-      <c r="X9" s="12" t="n">
+      <c r="X9" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Y9" s="12" t="n">
+      <c r="Y9" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z9" s="12" t="n">
+      <c r="Z9" s="28" t="n">
         <v>4.83</v>
       </c>
-      <c r="AA9" s="12" t="n">
+      <c r="AA9" s="28" t="n">
         <v>84.59999999999999</v>
       </c>
       <c r="AB9" s="8" t="n">
         <v>68</v>
       </c>
-      <c r="AC9" s="12" t="n">
+      <c r="AC9" s="28" t="n">
         <v>129</v>
       </c>
       <c r="AD9" s="8" t="n">
@@ -3656,13 +3995,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL9" s="13" t="inlineStr"/>
-      <c r="AM9" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN9" s="13" t="inlineStr">
+      <c r="AL9" s="29" t="inlineStr"/>
+      <c r="AM9" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN9" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -3680,22 +4019,25 @@
       <c r="AQ9" s="8" t="inlineStr"/>
       <c r="AR9" s="8" t="inlineStr"/>
       <c r="AS9" s="8" t="inlineStr"/>
-      <c r="AT9" s="8" t="inlineStr">
+      <c r="AT9" s="8" t="inlineStr"/>
+      <c r="AU9" s="8" t="inlineStr"/>
+      <c r="AV9" s="8" t="inlineStr"/>
+      <c r="AW9" s="8" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU9" s="13" t="inlineStr">
+      <c r="AX9" s="29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="AV9" s="13" t="inlineStr">
+      <c r="AY9" s="29" t="inlineStr">
         <is>
           <t>Budget edge but weak quiet-cove profile</t>
         </is>
       </c>
-      <c r="AW9" s="8" t="inlineStr">
+      <c r="AZ9" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -3755,13 +4097,13 @@
           <t>0.17375</t>
         </is>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="27" t="n">
         <v>930</v>
       </c>
-      <c r="M10" s="11" t="n">
+      <c r="M10" s="27" t="n">
         <v>465</v>
       </c>
-      <c r="N10" s="11" t="n">
+      <c r="N10" s="27" t="n">
         <v>66.43000000000001</v>
       </c>
       <c r="O10" s="8" t="inlineStr">
@@ -3780,37 +4122,37 @@
           <t>bungalow</t>
         </is>
       </c>
-      <c r="S10" s="12" t="n">
+      <c r="S10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="T10" s="12" t="n">
+      <c r="T10" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="U10" s="12" t="n">
+      <c r="U10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="V10" s="12" t="n">
+      <c r="V10" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="W10" s="12" t="n">
+      <c r="W10" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="X10" s="12" t="n">
+      <c r="X10" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="Y10" s="12" t="n">
+      <c r="Y10" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z10" s="12" t="n">
+      <c r="Z10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="AA10" s="12" t="n">
+      <c r="AA10" s="28" t="n">
         <v>98.40000000000001</v>
       </c>
       <c r="AB10" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="AC10" s="12" t="n">
+      <c r="AC10" s="28" t="n">
         <v>126.4</v>
       </c>
       <c r="AD10" s="8" t="n">
@@ -3851,13 +4193,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL10" s="13" t="inlineStr"/>
-      <c r="AM10" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN10" s="13" t="inlineStr">
+      <c r="AL10" s="29" t="inlineStr"/>
+      <c r="AM10" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN10" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -3875,22 +4217,25 @@
       <c r="AQ10" s="8" t="inlineStr"/>
       <c r="AR10" s="8" t="inlineStr"/>
       <c r="AS10" s="8" t="inlineStr"/>
-      <c r="AT10" s="8" t="inlineStr">
+      <c r="AT10" s="8" t="inlineStr"/>
+      <c r="AU10" s="8" t="inlineStr"/>
+      <c r="AV10" s="8" t="inlineStr"/>
+      <c r="AW10" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU10" s="13" t="inlineStr">
+      <c r="AX10" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV10" s="13" t="inlineStr">
+      <c r="AY10" s="29" t="inlineStr">
         <is>
           <t>Hard exclude despite good location</t>
         </is>
       </c>
-      <c r="AW10" s="8" t="inlineStr">
+      <c r="AZ10" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -3950,13 +4295,13 @@
           <t>-0.018617</t>
         </is>
       </c>
-      <c r="L11" s="11" t="n">
+      <c r="L11" s="27" t="n">
         <v>977.55</v>
       </c>
-      <c r="M11" s="11" t="n">
+      <c r="M11" s="27" t="n">
         <v>488.77</v>
       </c>
-      <c r="N11" s="11" t="n">
+      <c r="N11" s="27" t="n">
         <v>54.31</v>
       </c>
       <c r="O11" s="8" t="inlineStr">
@@ -3975,37 +4320,37 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S11" s="12" t="n">
+      <c r="S11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="12" t="n">
+      <c r="T11" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="U11" s="12" t="n">
+      <c r="U11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="V11" s="12" t="n">
+      <c r="V11" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="W11" s="12" t="n">
+      <c r="W11" s="28" t="n">
         <v>7.5</v>
       </c>
-      <c r="X11" s="12" t="n">
+      <c r="X11" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="Y11" s="12" t="n">
+      <c r="Y11" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z11" s="12" t="n">
+      <c r="Z11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="AA11" s="12" t="n">
+      <c r="AA11" s="28" t="n">
         <v>75.90000000000001</v>
       </c>
       <c r="AB11" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="AC11" s="12" t="n">
+      <c r="AC11" s="28" t="n">
         <v>125.8</v>
       </c>
       <c r="AD11" s="8" t="n">
@@ -4046,13 +4391,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL11" s="13" t="inlineStr"/>
-      <c r="AM11" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN11" s="13" t="inlineStr">
+      <c r="AL11" s="29" t="inlineStr"/>
+      <c r="AM11" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN11" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -4070,22 +4415,25 @@
       <c r="AQ11" s="8" t="inlineStr"/>
       <c r="AR11" s="8" t="inlineStr"/>
       <c r="AS11" s="8" t="inlineStr"/>
-      <c r="AT11" s="8" t="inlineStr">
+      <c r="AT11" s="8" t="inlineStr"/>
+      <c r="AU11" s="8" t="inlineStr"/>
+      <c r="AV11" s="8" t="inlineStr"/>
+      <c r="AW11" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU11" s="13" t="inlineStr">
+      <c r="AX11" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV11" s="13" t="inlineStr">
+      <c r="AY11" s="29" t="inlineStr">
         <is>
           <t>Hard exclude because child facility listed</t>
         </is>
       </c>
-      <c r="AW11" s="8" t="inlineStr">
+      <c r="AZ11" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -4145,13 +4493,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="L12" s="11" t="n">
+      <c r="L12" s="27" t="n">
         <v>1000</v>
       </c>
-      <c r="M12" s="11" t="n">
+      <c r="M12" s="27" t="n">
         <v>500</v>
       </c>
-      <c r="N12" s="11" t="n">
+      <c r="N12" s="27" t="n">
         <v>62.5</v>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -4174,31 +4522,31 @@
           <t>apartment</t>
         </is>
       </c>
-      <c r="S12" s="12" t="n">
+      <c r="S12" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="T12" s="12" t="n">
+      <c r="T12" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="U12" s="12" t="n">
+      <c r="U12" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="V12" s="12" t="n">
+      <c r="V12" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="W12" s="12" t="n">
+      <c r="W12" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="X12" s="12" t="n">
+      <c r="X12" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="Y12" s="12" t="n">
+      <c r="Y12" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="Z12" s="12" t="n">
+      <c r="Z12" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="AA12" s="12" t="inlineStr">
+      <c r="AA12" s="28" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -4208,7 +4556,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AC12" s="12" t="inlineStr">
+      <c r="AC12" s="28" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -4253,13 +4601,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL12" s="13" t="inlineStr"/>
-      <c r="AM12" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN12" s="13" t="inlineStr">
+      <c r="AL12" s="29" t="inlineStr"/>
+      <c r="AM12" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN12" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -4271,7 +4619,7 @@
       </c>
       <c r="AP12" s="8" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="AQ12" s="8" t="inlineStr">
@@ -4281,29 +4629,44 @@
       </c>
       <c r="AR12" s="8" t="inlineStr">
         <is>
+          <t>data/raw/link_01b1a36aa388.html</t>
+        </is>
+      </c>
+      <c r="AS12" s="8" t="inlineStr">
+        <is>
           <t>data/raw/link_01b1a36aa388.json</t>
         </is>
       </c>
-      <c r="AS12" s="8" t="inlineStr"/>
       <c r="AT12" s="8" t="inlineStr">
         <is>
+          <t>data/extracted/link_01b1a36aa388.json</t>
+        </is>
+      </c>
+      <c r="AU12" s="8" t="inlineStr">
+        <is>
+          <t>data/sheet-payloads/link_01b1a36aa388.json</t>
+        </is>
+      </c>
+      <c r="AV12" s="8" t="inlineStr"/>
+      <c r="AW12" s="8" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="AU12" s="13" t="inlineStr"/>
-      <c r="AV12" s="13" t="inlineStr">
+      <c r="AX12" s="29" t="inlineStr"/>
+      <c r="AY12" s="29" t="inlineStr">
         <is>
           <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
         </is>
       </c>
-      <c r="AW12" s="8" t="inlineStr">
+      <c r="AZ12" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW12"/>
+  <autoFilter ref="A1:AZ12"/>
   <conditionalFormatting sqref="Z2:Z12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -4336,7 +4699,7 @@
       <formula>"false"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT2:AT12">
+  <conditionalFormatting sqref="AW2:AW12">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
       <formula>"true"</formula>
     </cfRule>
@@ -4384,57 +4747,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>private_level</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>child_potential_0_10</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>quiet_score_0_10</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>beach_fit_0_10</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>transfer_score_0_10</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>budget_score_0_10</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>review_evidence_0_10</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>overall_score_0_10</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -4451,31 +4814,31 @@
           <t>Beniarbeig</t>
         </is>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="12" t="n">
+      <c r="E2" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="12" t="n">
+      <c r="F2" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="12" t="n">
+      <c r="G2" s="28" t="n">
         <v>6.5</v>
       </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="I2" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="12" t="n">
+      <c r="J2" s="28" t="n">
         <v>6.15</v>
       </c>
-      <c r="K2" s="13" t="inlineStr">
+      <c r="K2" s="29" t="inlineStr">
         <is>
           <t>Budget fit but inland and weak beach profile</t>
         </is>
@@ -4492,31 +4855,31 @@
           <t>Altea</t>
         </is>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="28" t="n">
         <v>7.4</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="G3" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="28" t="n">
         <v>6.83</v>
       </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="K3" s="29" t="inlineStr">
         <is>
           <t>Good Altea compromise but shared complex risk</t>
         </is>
@@ -4533,31 +4896,31 @@
           <t>Benitatxell Cumbre</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="28" t="n">
         <v>8.5</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="28" t="n">
         <v>7.22</v>
       </c>
-      <c r="K4" s="13" t="inlineStr">
+      <c r="K4" s="29" t="inlineStr">
         <is>
           <t>Best cove profile under 1000 EUR if 7 nights okay</t>
         </is>
@@ -4574,31 +4937,31 @@
           <t>Cumbre del Sol</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="28" t="n">
         <v>5.8</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="28" t="n">
         <v>7.8</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="28" t="n">
         <v>6.72</v>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="29" t="inlineStr">
         <is>
           <t>Strong Cumbre value but weak review evidence</t>
         </is>
@@ -4615,31 +4978,31 @@
           <t>Calp</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="28" t="n">
         <v>6.6</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="28" t="n">
         <v>7.2</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="28" t="n">
         <v>6.66</v>
       </c>
-      <c r="K6" s="13" t="inlineStr">
+      <c r="K6" s="29" t="inlineStr">
         <is>
           <t>Good price holiday home but only one review</t>
         </is>
@@ -4656,31 +5019,31 @@
           <t>Tarbena</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="28" t="n">
         <v>7.5</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="28" t="n">
         <v>6.96</v>
       </c>
-      <c r="K7" s="13" t="inlineStr">
+      <c r="K7" s="29" t="inlineStr">
         <is>
           <t>Quiet and under budget but inland not beach fit</t>
         </is>
@@ -4697,31 +5060,31 @@
           <t>Cumbre del Sol</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="28" t="n">
         <v>7.8</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="J8" s="12" t="n">
+      <c r="J8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="13" t="inlineStr">
+      <c r="K8" s="29" t="inlineStr">
         <is>
           <t>Good location but excluded by prior detail-risk evidence</t>
         </is>
@@ -4738,31 +5101,31 @@
           <t>Calp</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="28" t="n">
         <v>3.5</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="28" t="n">
         <v>4.83</v>
       </c>
-      <c r="K9" s="13" t="inlineStr">
+      <c r="K9" s="29" t="inlineStr">
         <is>
           <t>Budget edge but weak quiet-cove profile</t>
         </is>
@@ -4779,31 +5142,31 @@
           <t>Benitatxell</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H10" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="13" t="inlineStr">
+      <c r="K10" s="29" t="inlineStr">
         <is>
           <t>Hard exclude despite good location</t>
         </is>
@@ -4820,31 +5183,31 @@
           <t>Altea Hills</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="28" t="n">
         <v>7.5</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="K11" s="29" t="inlineStr">
         <is>
           <t>Hard exclude because child facility listed</t>
         </is>
@@ -4861,31 +5224,31 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="K12" s="13" t="inlineStr">
+      <c r="K12" s="29" t="inlineStr">
         <is>
           <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
         </is>
@@ -4930,7 +5293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW4"/>
+  <dimension ref="A1:AZ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4976,256 +5339,274 @@
     <col width="15" customWidth="1" min="41" max="41"/>
     <col width="21" customWidth="1" min="42" max="42"/>
     <col width="34" customWidth="1" min="43" max="43"/>
-    <col width="34" customWidth="1" min="44" max="44"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
     <col width="34" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
-    <col width="42" customWidth="1" min="48" max="48"/>
-    <col width="15" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="46" max="46"/>
+    <col width="21" customWidth="1" min="47" max="47"/>
+    <col width="34" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="19" customWidth="1" min="50" max="50"/>
+    <col width="42" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>date_range</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>nights</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>lng</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="26" t="inlineStr">
         <is>
           <t>price_total</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="26" t="inlineStr">
         <is>
           <t>price_per_person</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="26" t="inlineStr">
         <is>
           <t>price_per_person_per_night</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="26" t="inlineStr">
         <is>
           <t>budget_under_500pp</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="P1" s="26" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="Q1" s="26" t="inlineStr">
         <is>
           <t>review_count</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="R1" s="26" t="inlineStr">
         <is>
           <t>property_type</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="S1" s="26" t="inlineStr">
         <is>
           <t>private_level</t>
         </is>
       </c>
-      <c r="T1" s="10" t="inlineStr">
+      <c r="T1" s="26" t="inlineStr">
         <is>
           <t>child_potential_0_10</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="U1" s="26" t="inlineStr">
         <is>
           <t>quiet_score_0_10</t>
         </is>
       </c>
-      <c r="V1" s="10" t="inlineStr">
+      <c r="V1" s="26" t="inlineStr">
         <is>
           <t>review_evidence_0_10</t>
         </is>
       </c>
-      <c r="W1" s="10" t="inlineStr">
+      <c r="W1" s="26" t="inlineStr">
         <is>
           <t>beach_fit_0_10</t>
         </is>
       </c>
-      <c r="X1" s="10" t="inlineStr">
+      <c r="X1" s="26" t="inlineStr">
         <is>
           <t>transfer_score_0_10</t>
         </is>
       </c>
-      <c r="Y1" s="10" t="inlineStr">
+      <c r="Y1" s="26" t="inlineStr">
         <is>
           <t>budget_score_0_10</t>
         </is>
       </c>
-      <c r="Z1" s="10" t="inlineStr">
+      <c r="Z1" s="26" t="inlineStr">
         <is>
           <t>overall_score_0_10</t>
         </is>
       </c>
-      <c r="AA1" s="10" t="inlineStr">
+      <c r="AA1" s="26" t="inlineStr">
         <is>
           <t>alc_km_est</t>
         </is>
       </c>
-      <c r="AB1" s="10" t="inlineStr">
+      <c r="AB1" s="26" t="inlineStr">
         <is>
           <t>alc_drive_min_est</t>
         </is>
       </c>
-      <c r="AC1" s="10" t="inlineStr">
+      <c r="AC1" s="26" t="inlineStr">
         <is>
           <t>vlc_km_est</t>
         </is>
       </c>
-      <c r="AD1" s="10" t="inlineStr">
+      <c r="AD1" s="26" t="inlineStr">
         <is>
           <t>vlc_drive_min_est</t>
         </is>
       </c>
-      <c r="AE1" s="10" t="inlineStr">
+      <c r="AE1" s="26" t="inlineStr">
         <is>
           <t>airport_distance_method</t>
         </is>
       </c>
-      <c r="AF1" s="10" t="inlineStr">
+      <c r="AF1" s="26" t="inlineStr">
         <is>
           <t>pool_type</t>
         </is>
       </c>
-      <c r="AG1" s="10" t="inlineStr">
+      <c r="AG1" s="26" t="inlineStr">
         <is>
           <t>whole_place_evidence</t>
         </is>
       </c>
-      <c r="AH1" s="10" t="inlineStr">
+      <c r="AH1" s="26" t="inlineStr">
         <is>
           <t>kitchen</t>
         </is>
       </c>
-      <c r="AI1" s="10" t="inlineStr">
+      <c r="AI1" s="26" t="inlineStr">
         <is>
           <t>air_conditioning</t>
         </is>
       </c>
-      <c r="AJ1" s="10" t="inlineStr">
+      <c r="AJ1" s="26" t="inlineStr">
         <is>
           <t>parking</t>
         </is>
       </c>
-      <c r="AK1" s="10" t="inlineStr">
+      <c r="AK1" s="26" t="inlineStr">
         <is>
           <t>terrace_or_balcony</t>
         </is>
       </c>
-      <c r="AL1" s="10" t="inlineStr">
+      <c r="AL1" s="26" t="inlineStr">
         <is>
           <t>family_red_flags</t>
         </is>
       </c>
-      <c r="AM1" s="10" t="inlineStr">
+      <c r="AM1" s="26" t="inlineStr">
         <is>
           <t>quiet_evidence</t>
         </is>
       </c>
-      <c r="AN1" s="10" t="inlineStr">
+      <c r="AN1" s="26" t="inlineStr">
         <is>
           <t>review_evidence</t>
         </is>
       </c>
-      <c r="AO1" s="10" t="inlineStr">
+      <c r="AO1" s="26" t="inlineStr">
         <is>
           <t>crawl_status</t>
         </is>
       </c>
-      <c r="AP1" s="10" t="inlineStr">
+      <c r="AP1" s="26" t="inlineStr">
         <is>
           <t>needs_manual_input</t>
         </is>
       </c>
-      <c r="AQ1" s="10" t="inlineStr">
+      <c r="AQ1" s="26" t="inlineStr">
         <is>
           <t>raw_markdown_path</t>
         </is>
       </c>
-      <c r="AR1" s="10" t="inlineStr">
+      <c r="AR1" s="26" t="inlineStr">
+        <is>
+          <t>raw_html_path</t>
+        </is>
+      </c>
+      <c r="AS1" s="26" t="inlineStr">
         <is>
           <t>raw_json_path</t>
         </is>
       </c>
-      <c r="AS1" s="10" t="inlineStr">
+      <c r="AT1" s="26" t="inlineStr">
+        <is>
+          <t>extracted_json_path</t>
+        </is>
+      </c>
+      <c r="AU1" s="26" t="inlineStr">
+        <is>
+          <t>sheet_payload_path</t>
+        </is>
+      </c>
+      <c r="AV1" s="26" t="inlineStr">
         <is>
           <t>screenshot_path</t>
         </is>
       </c>
-      <c r="AT1" s="10" t="inlineStr">
+      <c r="AW1" s="26" t="inlineStr">
         <is>
           <t>excluded</t>
         </is>
       </c>
-      <c r="AU1" s="10" t="inlineStr">
+      <c r="AX1" s="26" t="inlineStr">
         <is>
           <t>exclusion_reason</t>
         </is>
       </c>
-      <c r="AV1" s="10" t="inlineStr">
+      <c r="AY1" s="26" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="AW1" s="10" t="inlineStr">
+      <c r="AZ1" s="26" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5381,13 +5762,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL2" s="13" t="inlineStr"/>
-      <c r="AM2" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN2" s="13" t="inlineStr">
+      <c r="AL2" s="29" t="inlineStr"/>
+      <c r="AM2" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN2" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -5405,22 +5786,25 @@
       <c r="AQ2" s="8" t="inlineStr"/>
       <c r="AR2" s="8" t="inlineStr"/>
       <c r="AS2" s="8" t="inlineStr"/>
-      <c r="AT2" s="8" t="inlineStr">
+      <c r="AT2" s="8" t="inlineStr"/>
+      <c r="AU2" s="8" t="inlineStr"/>
+      <c r="AV2" s="8" t="inlineStr"/>
+      <c r="AW2" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU2" s="13" t="inlineStr">
+      <c r="AX2" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV2" s="13" t="inlineStr">
+      <c r="AY2" s="29" t="inlineStr">
         <is>
           <t>Good location but excluded by prior detail-risk evidence</t>
         </is>
       </c>
-      <c r="AW2" s="8" t="inlineStr">
+      <c r="AZ2" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -5576,13 +5960,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL3" s="13" t="inlineStr"/>
-      <c r="AM3" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN3" s="13" t="inlineStr">
+      <c r="AL3" s="29" t="inlineStr"/>
+      <c r="AM3" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN3" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -5600,22 +5984,25 @@
       <c r="AQ3" s="8" t="inlineStr"/>
       <c r="AR3" s="8" t="inlineStr"/>
       <c r="AS3" s="8" t="inlineStr"/>
-      <c r="AT3" s="8" t="inlineStr">
+      <c r="AT3" s="8" t="inlineStr"/>
+      <c r="AU3" s="8" t="inlineStr"/>
+      <c r="AV3" s="8" t="inlineStr"/>
+      <c r="AW3" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU3" s="13" t="inlineStr">
+      <c r="AX3" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV3" s="13" t="inlineStr">
+      <c r="AY3" s="29" t="inlineStr">
         <is>
           <t>Hard exclude despite good location</t>
         </is>
       </c>
-      <c r="AW3" s="8" t="inlineStr">
+      <c r="AZ3" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -5771,13 +6158,13 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AL4" s="13" t="inlineStr"/>
-      <c r="AM4" s="13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN4" s="13" t="inlineStr">
+      <c r="AL4" s="29" t="inlineStr"/>
+      <c r="AM4" s="29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN4" s="29" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
@@ -5795,29 +6182,32 @@
       <c r="AQ4" s="8" t="inlineStr"/>
       <c r="AR4" s="8" t="inlineStr"/>
       <c r="AS4" s="8" t="inlineStr"/>
-      <c r="AT4" s="8" t="inlineStr">
+      <c r="AT4" s="8" t="inlineStr"/>
+      <c r="AU4" s="8" t="inlineStr"/>
+      <c r="AV4" s="8" t="inlineStr"/>
+      <c r="AW4" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AU4" s="13" t="inlineStr">
+      <c r="AX4" s="29" t="inlineStr">
         <is>
           <t>family_no_go</t>
         </is>
       </c>
-      <c r="AV4" s="13" t="inlineStr">
+      <c r="AY4" s="29" t="inlineStr">
         <is>
           <t>Hard exclude because child facility listed</t>
         </is>
       </c>
-      <c r="AW4" s="8" t="inlineStr">
+      <c r="AZ4" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW4"/>
+  <autoFilter ref="A1:AZ4"/>
   <conditionalFormatting sqref="Z2:Z4">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -5850,7 +6240,7 @@
       <formula>"false"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AT2:AT4">
+  <conditionalFormatting sqref="AW2:AW4">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
       <formula>"true"</formula>
     </cfRule>
@@ -5883,22 +6273,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Airport</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>Rolle</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>Notiz</t>
         </is>
@@ -5981,62 +6371,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>link_id</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>submitted_by</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>date_range_hint</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>crawl_status</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>needs_manual_input</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>reviewed</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="26" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -6057,7 +6447,7 @@
       <c r="D2" s="8" t="inlineStr"/>
       <c r="E2" s="8" t="inlineStr"/>
       <c r="F2" s="8" t="inlineStr"/>
-      <c r="G2" s="13" t="inlineStr"/>
+      <c r="G2" s="29" t="inlineStr"/>
       <c r="H2" s="8" t="inlineStr"/>
       <c r="I2" s="8" t="inlineStr"/>
       <c r="J2" s="8" t="inlineStr">
@@ -6091,7 +6481,7 @@
       <c r="D3" s="8" t="inlineStr"/>
       <c r="E3" s="8" t="inlineStr"/>
       <c r="F3" s="8" t="inlineStr"/>
-      <c r="G3" s="13" t="inlineStr"/>
+      <c r="G3" s="29" t="inlineStr"/>
       <c r="H3" s="8" t="inlineStr"/>
       <c r="I3" s="8" t="inlineStr"/>
       <c r="J3" s="8" t="inlineStr">
@@ -6141,7 +6531,7 @@
           <t>8 nights, user note: ca. 500 EUR pp</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="29" t="inlineStr">
         <is>
           <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights.</t>
         </is>
@@ -6196,17 +6586,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Komponente</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="30" t="inlineStr">
         <is>
           <t>Gewicht</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="30" t="inlineStr">
         <is>
           <t>Logik</t>
         </is>
@@ -6359,7 +6749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6368,65 +6758,83 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>crawl_status</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>needs_manual_input</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>raw_markdown_path</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>raw_html_path</t>
+        </is>
+      </c>
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>raw_json_path</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
+        <is>
+          <t>extracted_json_path</t>
+        </is>
+      </c>
+      <c r="J1" s="26" t="inlineStr">
+        <is>
+          <t>sheet_payload_path</t>
+        </is>
+      </c>
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>screenshot_path</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="L1" s="26" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="M1" s="26" t="inlineStr">
         <is>
           <t>link_id</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="N1" s="26" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -6461,13 +6869,16 @@
       <c r="F2" s="8" t="inlineStr"/>
       <c r="G2" s="8" t="inlineStr"/>
       <c r="H2" s="8" t="inlineStr"/>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I2" s="8" t="inlineStr"/>
       <c r="J2" s="8" t="inlineStr"/>
       <c r="K2" s="8" t="inlineStr"/>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr"/>
+      <c r="N2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -6498,13 +6909,16 @@
       <c r="F3" s="8" t="inlineStr"/>
       <c r="G3" s="8" t="inlineStr"/>
       <c r="H3" s="8" t="inlineStr"/>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I3" s="8" t="inlineStr"/>
       <c r="J3" s="8" t="inlineStr"/>
       <c r="K3" s="8" t="inlineStr"/>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr"/>
+      <c r="N3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -6535,13 +6949,16 @@
       <c r="F4" s="8" t="inlineStr"/>
       <c r="G4" s="8" t="inlineStr"/>
       <c r="H4" s="8" t="inlineStr"/>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I4" s="8" t="inlineStr"/>
       <c r="J4" s="8" t="inlineStr"/>
       <c r="K4" s="8" t="inlineStr"/>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr"/>
+      <c r="N4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -6572,13 +6989,16 @@
       <c r="F5" s="8" t="inlineStr"/>
       <c r="G5" s="8" t="inlineStr"/>
       <c r="H5" s="8" t="inlineStr"/>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I5" s="8" t="inlineStr"/>
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="8" t="inlineStr"/>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr"/>
+      <c r="N5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -6609,13 +7029,16 @@
       <c r="F6" s="8" t="inlineStr"/>
       <c r="G6" s="8" t="inlineStr"/>
       <c r="H6" s="8" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I6" s="8" t="inlineStr"/>
       <c r="J6" s="8" t="inlineStr"/>
       <c r="K6" s="8" t="inlineStr"/>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr"/>
+      <c r="N6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -6646,13 +7069,16 @@
       <c r="F7" s="8" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr"/>
       <c r="H7" s="8" t="inlineStr"/>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I7" s="8" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="8" t="inlineStr"/>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr"/>
+      <c r="N7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -6683,13 +7109,16 @@
       <c r="F8" s="8" t="inlineStr"/>
       <c r="G8" s="8" t="inlineStr"/>
       <c r="H8" s="8" t="inlineStr"/>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I8" s="8" t="inlineStr"/>
       <c r="J8" s="8" t="inlineStr"/>
       <c r="K8" s="8" t="inlineStr"/>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr"/>
+      <c r="N8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -6720,13 +7149,16 @@
       <c r="F9" s="8" t="inlineStr"/>
       <c r="G9" s="8" t="inlineStr"/>
       <c r="H9" s="8" t="inlineStr"/>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I9" s="8" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr"/>
       <c r="K9" s="8" t="inlineStr"/>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr"/>
+      <c r="N9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -6757,13 +7189,16 @@
       <c r="F10" s="8" t="inlineStr"/>
       <c r="G10" s="8" t="inlineStr"/>
       <c r="H10" s="8" t="inlineStr"/>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I10" s="8" t="inlineStr"/>
       <c r="J10" s="8" t="inlineStr"/>
       <c r="K10" s="8" t="inlineStr"/>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr"/>
+      <c r="N10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -6794,13 +7229,16 @@
       <c r="F11" s="8" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr"/>
       <c r="H11" s="8" t="inlineStr"/>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="I11" s="8" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr"/>
       <c r="K11" s="8" t="inlineStr"/>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr"/>
+      <c r="N11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -6825,7 +7263,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -6835,17 +7273,32 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
+          <t>data/raw/link_01b1a36aa388.html</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
           <t>data/raw/link_01b1a36aa388.json</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr"/>
       <c r="I12" s="8" t="inlineStr">
         <is>
+          <t>data/extracted/link_01b1a36aa388.json</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>data/sheet-payloads/link_01b1a36aa388.json</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr"/>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr"/>
-      <c r="K12" s="8" t="inlineStr"/>
+      <c r="M12" s="8" t="inlineStr"/>
+      <c r="N12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr"/>
@@ -6860,13 +7313,16 @@
       <c r="F13" s="8" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr"/>
       <c r="H13" s="8" t="inlineStr"/>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr"/>
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr"/>
-      <c r="K13" s="8" t="inlineStr">
+      <c r="M13" s="8" t="inlineStr"/>
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>new</t>
         </is>
@@ -6885,13 +7341,16 @@
       <c r="F14" s="8" t="inlineStr"/>
       <c r="G14" s="8" t="inlineStr"/>
       <c r="H14" s="8" t="inlineStr"/>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr"/>
+      <c r="K14" s="8" t="inlineStr"/>
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr"/>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr"/>
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>new</t>
         </is>
@@ -6918,24 +7377,27 @@
       <c r="F15" s="8" t="inlineStr"/>
       <c r="G15" s="8" t="inlineStr"/>
       <c r="H15" s="8" t="inlineStr"/>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr"/>
+      <c r="J15" s="8" t="inlineStr"/>
+      <c r="K15" s="8" t="inlineStr"/>
+      <c r="L15" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>link_01b1a36aa388</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K15"/>
+  <autoFilter ref="A1:N15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>

</xml_diff>

<commit_message>
Update travel candidates from link intake
</commit_message>
<xml_diff>
--- a/exports/costa-blanca-matrix.xlsx
+++ b/exports/costa-blanca-matrix.xlsx
@@ -906,7 +906,7 @@
       </c>
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="4" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="n"/>
     </row>
@@ -1515,29 +1515,21 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Can Lluna</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Tarbena</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>466.38</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>6.96</v>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>9</v>
-      </c>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr"/>
+      <c r="D32" s="8" t="inlineStr"/>
+      <c r="E32" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/es/can-lluna.html</t>
+          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
         </is>
       </c>
       <c r="H32" s="2" t="n"/>
@@ -1545,29 +1537,29 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Apartment mit Blick auf das Mittelmeer</t>
+          <t>Can Lluna</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>Tarbena</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>500</v>
+        <v>466.38</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>5.5</v>
+        <v>6.96</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>1.5</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>https://www.airbnb.de/rooms/1202192166783165853?unique_share_id=ddf4638d-cc1a-4792-abed-520d6373d0d5&amp;viralityEntryPoint=1&amp;s=76</t>
+          <t>https://www.booking.com/hotel/es/can-lluna.html</t>
         </is>
       </c>
       <c r="H33" s="2" t="n"/>
@@ -2039,7 +2031,7 @@
       <c r="B55" s="8" t="n"/>
       <c r="C55" s="8" t="n"/>
       <c r="D55" s="25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
@@ -2071,7 +2063,7 @@
       <c r="B57" s="8" t="n"/>
       <c r="C57" s="8" t="n"/>
       <c r="D57" s="25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
@@ -4447,7 +4439,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>candidate</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -4462,7 +4454,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Apartment mit Blick auf das Mittelmeer</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -4472,7 +4464,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>8 nights (user-provided)</t>
+          <t>8 nights, user note: ca. 500 EUR pp</t>
         </is>
       </c>
       <c r="H12" s="8" t="n">
@@ -4483,145 +4475,51 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="L12" s="27" t="n">
-        <v>1000</v>
-      </c>
-      <c r="M12" s="27" t="n">
-        <v>500</v>
-      </c>
-      <c r="N12" s="27" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr"/>
+      <c r="L12" s="27" t="inlineStr"/>
+      <c r="M12" s="27" t="inlineStr"/>
+      <c r="N12" s="27" t="inlineStr"/>
+      <c r="O12" s="8" t="inlineStr"/>
+      <c r="P12" s="8" t="inlineStr"/>
+      <c r="Q12" s="8" t="inlineStr"/>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S12" s="28" t="inlineStr"/>
+      <c r="T12" s="28" t="inlineStr"/>
+      <c r="U12" s="28" t="inlineStr"/>
+      <c r="V12" s="28" t="inlineStr"/>
+      <c r="W12" s="28" t="inlineStr"/>
+      <c r="X12" s="28" t="inlineStr"/>
+      <c r="Y12" s="28" t="inlineStr"/>
+      <c r="Z12" s="28" t="inlineStr"/>
+      <c r="AA12" s="28" t="inlineStr"/>
+      <c r="AB12" s="8" t="inlineStr"/>
+      <c r="AC12" s="28" t="inlineStr"/>
+      <c r="AD12" s="8" t="inlineStr"/>
+      <c r="AE12" s="8" t="inlineStr"/>
+      <c r="AF12" s="8" t="inlineStr"/>
+      <c r="AG12" s="8" t="inlineStr"/>
+      <c r="AH12" s="8" t="inlineStr"/>
+      <c r="AI12" s="8" t="inlineStr"/>
+      <c r="AJ12" s="8" t="inlineStr"/>
+      <c r="AK12" s="8" t="inlineStr"/>
+      <c r="AL12" s="29" t="inlineStr"/>
+      <c r="AM12" s="29" t="inlineStr"/>
+      <c r="AN12" s="29" t="inlineStr"/>
+      <c r="AO12" s="8" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="AP12" s="8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="Q12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="R12" s="8" t="inlineStr">
-        <is>
-          <t>apartment</t>
-        </is>
-      </c>
-      <c r="S12" s="28" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="T12" s="28" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="U12" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="V12" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="W12" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="X12" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y12" s="28" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z12" s="28" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="AA12" s="28" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AB12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AC12" s="28" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AD12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AE12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AF12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AH12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AI12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AJ12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AK12" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AL12" s="29" t="inlineStr"/>
-      <c r="AM12" s="29" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AN12" s="29" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AO12" s="8" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AP12" s="8" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
       <c r="AQ12" s="8" t="inlineStr">
         <is>
           <t>data/raw/link_01b1a36aa388.md</t>
@@ -4637,11 +4535,7 @@
           <t>data/raw/link_01b1a36aa388.json</t>
         </is>
       </c>
-      <c r="AT12" s="8" t="inlineStr">
-        <is>
-          <t>data/extracted/link_01b1a36aa388.json</t>
-        </is>
-      </c>
+      <c r="AT12" s="8" t="inlineStr"/>
       <c r="AU12" s="8" t="inlineStr">
         <is>
           <t>data/sheet-payloads/link_01b1a36aa388.json</t>
@@ -4656,7 +4550,7 @@
       <c r="AX12" s="29" t="inlineStr"/>
       <c r="AY12" s="29" t="inlineStr">
         <is>
-          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
+          <t>Re-run requested via ChatGPT on 2026-07-02. If location, exact dates, price or reviews remain unknown, manual validation is required.</t>
         </is>
       </c>
       <c r="AZ12" s="8" t="inlineStr">
@@ -5216,7 +5110,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Apartment mit Blick auf das Mittelmeer</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -5224,33 +5118,17 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="D12" s="28" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="H12" s="28" t="n">
-        <v>7</v>
-      </c>
-      <c r="I12" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="28" t="n">
-        <v>5.5</v>
-      </c>
+      <c r="C12" s="28" t="inlineStr"/>
+      <c r="D12" s="28" t="inlineStr"/>
+      <c r="E12" s="28" t="inlineStr"/>
+      <c r="F12" s="28" t="inlineStr"/>
+      <c r="G12" s="28" t="inlineStr"/>
+      <c r="H12" s="28" t="inlineStr"/>
+      <c r="I12" s="28" t="inlineStr"/>
+      <c r="J12" s="28" t="inlineStr"/>
       <c r="K12" s="29" t="inlineStr">
         <is>
-          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights. Price/nights entered from user note; location still needs manual confirmation.</t>
+          <t>Re-run requested via ChatGPT on 2026-07-02. If location, exact dates, price or reviews remain unknown, manual validation is required.</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6386,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -6533,7 +6411,7 @@
       </c>
       <c r="G4" s="29" t="inlineStr">
         <is>
-          <t>User flagged as strong price find: ca. 500 EUR per person for 8 nights.</t>
+          <t>Re-run requested via ChatGPT on 2026-07-02. If location, exact dates, price or reviews remain unknown, manual validation is required.</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
@@ -6543,12 +6421,12 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
@@ -7248,7 +7126,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Apartment mit Blick auf das Mittelmeer</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -7258,12 +7136,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -7281,11 +7159,7 @@
           <t>data/raw/link_01b1a36aa388.json</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>data/extracted/link_01b1a36aa388.json</t>
-        </is>
-      </c>
+      <c r="I12" s="8" t="inlineStr"/>
       <c r="J12" s="8" t="inlineStr">
         <is>
           <t>data/sheet-payloads/link_01b1a36aa388.json</t>
@@ -7366,12 +7240,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr"/>
@@ -7392,7 +7266,7 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>failed</t>
         </is>
       </c>
     </row>

</xml_diff>